<commit_message>
added fa page, enabled form
</commit_message>
<xml_diff>
--- a/server/data/products.xlsx
+++ b/server/data/products.xlsx
@@ -436,10 +436,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Hogwarts House Crest Desk Stand</v>
+        <v>House Sigil Desk Monument</v>
       </c>
       <c r="C2" t="str">
-        <v>Laser-cut wooden desk stand featuring your Hogwarts house crest. Choose from Gryffindor, Slytherin, Ravenclaw, or Hufflepuff. Perfect for Potterheads.</v>
+        <v>Four ancient houses. One choice that defines you. Laser-cut wooden monument featuring your chosen sigil. For those who know that where you belong matters more than where you started. Precision-crafted in Jaipur.</v>
       </c>
       <c r="D2">
         <v>899</v>
@@ -448,13 +448,13 @@
         <v>Birch Wood</v>
       </c>
       <c r="F2" t="str">
-        <v>Display your Hogwarts house pride on your desk. Great gift for Harry Potter fans.</v>
+        <v>Declare your allegiance. Symbol of wisdom, courage, ambition, or loyalty - your desk, your manifesto.</v>
       </c>
       <c r="G2" t="str">
         <v>Collectibles</v>
       </c>
       <c r="H2" t="str">
-        <v>https://placeholder-image-url.com/hogwarts-crest.jpg</v>
+        <v>https://placeholder-image-url.com/house-sigil.jpg</v>
       </c>
       <c r="I2" t="str">
         <v>15cm x 12cm x 3cm</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Iron Man Arc Reactor Phone Stand</v>
+        <v>Arc Emblem Phone Stand</v>
       </c>
       <c r="C3" t="str">
-        <v>3D-printed phone stand inspired by Iron Man's arc reactor design. Holds your phone at the perfect viewing angle.</v>
+        <v>3D-printed phone stand inspired by genius engineering. Power symbol in circular precision. Holds your device at the perfect angle. For those who know innovation is identity.</v>
       </c>
       <c r="D3">
         <v>749</v>
@@ -480,13 +480,13 @@
         <v>PLA Plastic</v>
       </c>
       <c r="F3" t="str">
-        <v>For Marvel fans who want to power up their desk with Stark tech aesthetics.</v>
+        <v>Your workspace, powered by the same energy that drives visionaries. Precision-cut in Jaipur.</v>
       </c>
       <c r="G3" t="str">
         <v>Desk Accessories</v>
       </c>
       <c r="H3" t="str">
-        <v>https://placeholder-image-url.com/arc-reactor.jpg</v>
+        <v>https://placeholder-image-url.com/arc-emblem.jpg</v>
       </c>
       <c r="I3" t="str">
         <v>12cm x 10cm x 8cm</v>
@@ -500,10 +500,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Lightsaber Pen Holder</v>
+        <v>Dueling Relic Pen Holder</v>
       </c>
       <c r="C4" t="str">
-        <v>Laser-cut acrylic pen holder shaped like an iconic lightsaber hilt. Choose your side: Jedi blue or Sith red.</v>
+        <v>Laser-cut acrylic pen holder shaped like an elegant weapon hilt. Choose your allegiance: guardian blue or defiant red. Ancient conflicts, modern desk. The Force is not fiction - it is philosophy.</v>
       </c>
       <c r="D4">
         <v>649</v>
@@ -512,13 +512,13 @@
         <v>Colored Acrylic</v>
       </c>
       <c r="F4" t="str">
-        <v>Store your pens, pencils, and markers in this Star Wars inspired holder. May the Force be with your stationery.</v>
+        <v>Store your tools in a symbol of cosmic balance. Light or dark - your choice, your identity.</v>
       </c>
       <c r="G4" t="str">
         <v>Desk Accessories</v>
       </c>
       <c r="H4" t="str">
-        <v>https://placeholder-image-url.com/lightsaber.jpg</v>
+        <v>https://placeholder-image-url.com/dueling-relic.jpg</v>
       </c>
       <c r="I4" t="str">
         <v>20cm x 5cm x 5cm</v>
@@ -532,10 +532,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Personalized Wizard Name Plate</v>
+        <v>Cosmic Script Name Plate</v>
       </c>
       <c r="C5" t="str">
-        <v>Laser-cut wooden name plate with your name in a magical font, complete with star accents. Custom engraving included.</v>
+        <v>Laser-cut wooden name plate with your name in an otherworldly font, complete with star accents. Custom engraving. Professional, yet subtly extraordinary. Crafted in Jaipur.</v>
       </c>
       <c r="D5">
         <v>599</v>
@@ -544,13 +544,13 @@
         <v>Walnut Wood</v>
       </c>
       <c r="F5" t="str">
-        <v>Professional yet magical desk nameplate. Perfect for Potterheads in the workplace.</v>
+        <v>Your name, your desk, your universe. For those who bring magic to the mundane without explanation.</v>
       </c>
       <c r="G5" t="str">
         <v>Gifts</v>
       </c>
       <c r="H5" t="str">
-        <v>https://placeholder-image-url.com/wizard-nameplate.jpg</v>
+        <v>https://placeholder-image-url.com/cosmic-nameplate.jpg</v>
       </c>
       <c r="I5" t="str">
         <v>22cm x 6cm x 1.5cm</v>
@@ -564,10 +564,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>Marvel Avengers Coaster Set</v>
+        <v>Hero Emblems Coaster Set</v>
       </c>
       <c r="C6" t="str">
-        <v>Set of 4 laser-cut wooden coasters featuring iconic Avengers symbols: Iron Man, Captain America, Thor, and Hulk.</v>
+        <v>Set of 4 laser-cut wooden coasters featuring iconic superhero symbols. Shield, arc, lightning, strength. Protect your desk surface while quietly declaring allegiance to extraordinary ideals.</v>
       </c>
       <c r="D6">
         <v>499</v>
@@ -576,13 +576,13 @@
         <v>Bamboo Wood</v>
       </c>
       <c r="F6" t="str">
-        <v>Protect your desk surface while showing your Marvel allegiance. Great gift for Avengers fans.</v>
+        <v>Not all heroes wear capes. Some just have impeccable desk aesthetics. Indian-crafted precision.</v>
       </c>
       <c r="G6" t="str">
         <v>Desk Accessories</v>
       </c>
       <c r="H6" t="str">
-        <v>https://placeholder-image-url.com/avengers-coasters.jpg</v>
+        <v>https://placeholder-image-url.com/hero-emblems.jpg</v>
       </c>
       <c r="I6" t="str">
         <v>10cm diameter x 0.8cm (each)</v>
@@ -596,10 +596,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>Baby Yoda (Grogu) Desk Buddy</v>
+        <v>Small Guardian Desk Companion</v>
       </c>
       <c r="C7" t="str">
-        <v>3D-printed Grogu figurine for your desk. Adorable design with precise detailing. The Child will watch over your work.</v>
+        <v>3D-printed desk companion with large, knowing eyes. Adorable design with precise detailing. Watches over your workspace with ancient wisdom in tiny form. This is the way.</v>
       </c>
       <c r="D7">
         <v>999</v>
@@ -608,13 +608,13 @@
         <v>PLA Plastic</v>
       </c>
       <c r="F7" t="str">
-        <v>Desk companion for Mandalorian fans. This is the way to decorate your workspace.</v>
+        <v>Desk guardian for those who understand that the most powerful often come in unexpected packages.</v>
       </c>
       <c r="G7" t="str">
         <v>Collectibles</v>
       </c>
       <c r="H7" t="str">
-        <v>https://placeholder-image-url.com/grogu.jpg</v>
+        <v>https://placeholder-image-url.com/guardian.jpg</v>
       </c>
       <c r="I7" t="str">
         <v>10cm x 6cm x 6cm</v>
@@ -628,10 +628,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>Sorting Hat Pen Stand</v>
+        <v>Wisdom Keeper Pen Stand</v>
       </c>
       <c r="C8" t="str">
-        <v>3D-printed replica of the Hogwarts Sorting Hat that holds your pens. Detailed texture and weathered finish.</v>
+        <v>3D-printed replica of an ancient sorting artifact that holds your pens. Detailed texture and weathered finish. Let destiny decide where your tools belong.</v>
       </c>
       <c r="D8">
         <v>849</v>
@@ -640,13 +640,13 @@
         <v>PLA Plastic</v>
       </c>
       <c r="F8" t="str">
-        <v>Let the Sorting Hat sort your stationery. Perfect for any Potterhead's desk.</v>
+        <v>Organize your stationery with the same wisdom that sorts souls. Crafted in Jaipur workshops.</v>
       </c>
       <c r="G8" t="str">
         <v>Desk Accessories</v>
       </c>
       <c r="H8" t="str">
-        <v>https://placeholder-image-url.com/sorting-hat.jpg</v>
+        <v>https://placeholder-image-url.com/wisdom-keeper.jpg</v>
       </c>
       <c r="I8" t="str">
         <v>12cm x 12cm x 10cm</v>
@@ -660,10 +660,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Spider-Man Web Shooter Cable Organizer</v>
+        <v>Arachnid Web Cable Organizer</v>
       </c>
       <c r="C9" t="str">
-        <v>3D-printed cable holder inspired by Spider-Man's web shooters. Keeps your desk cables tangle-free in heroic style.</v>
+        <v>3D-printed cable holder inspired by bio-mechanical precision. Keeps your desk cables tangle-free with spider-like efficiency. With great organization comes great productivity.</v>
       </c>
       <c r="D9">
         <v>449</v>
@@ -672,13 +672,13 @@
         <v>PLA Plastic</v>
       </c>
       <c r="F9" t="str">
-        <v>Swing into organization with this Spider-Man inspired desk accessory. Set of 2.</v>
+        <v>Web-slinging cable management for those who swing between chaos and control. Set of 2.</v>
       </c>
       <c r="G9" t="str">
         <v>Desk Accessories</v>
       </c>
       <c r="H9" t="str">
-        <v>https://placeholder-image-url.com/web-shooter.jpg</v>
+        <v>https://placeholder-image-url.com/web-organizer.jpg</v>
       </c>
       <c r="I9" t="str">
         <v>6cm x 4cm x 3cm (each)</v>
@@ -692,10 +692,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Deathly Hallows Bookmark</v>
+        <v>Hallowed Symbols Bookmark</v>
       </c>
       <c r="C10" t="str">
-        <v>Laser-cut wooden bookmark featuring the iconic Deathly Hallows symbol. Elegant and meaningful.</v>
+        <v>Laser-cut wooden bookmark featuring the trinity of ancient relics. Elegant and meaningful. Three objects, one master of death. Mark your place in stories that matter.</v>
       </c>
       <c r="D10">
         <v>249</v>
@@ -704,13 +704,13 @@
         <v>Walnut Wood</v>
       </c>
       <c r="F10" t="str">
-        <v>Mark your place in your favorite books with this Harry Potter inspired bookmark. Perfect gift for readers.</v>
+        <v>For readers who know that some symbols hold more power than words. Indian-crafted precision.</v>
       </c>
       <c r="G10" t="str">
         <v>Gifts</v>
       </c>
       <c r="H10" t="str">
-        <v>https://placeholder-image-url.com/deathly-hallows.jpg</v>
+        <v>https://placeholder-image-url.com/hallowed-symbols.jpg</v>
       </c>
       <c r="I10" t="str">
         <v>15cm x 4cm x 0.3cm</v>
@@ -724,10 +724,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Flexi Dragon (Game of Thrones Inspired)</v>
+        <v>Articulated Mythic Serpent</v>
       </c>
       <c r="C11" t="str">
-        <v>3D-printed articulated dragon figure with movable wings and body. Fully poseable with smooth joints.</v>
+        <v>3D-printed articulated creature with movable wings and body. Fully poseable with smooth joints. Fantasy made tangible. Fire and flight in flexible form.</v>
       </c>
       <c r="D11">
         <v>999</v>
@@ -736,13 +736,13 @@
         <v>TPU Flexible Plastic</v>
       </c>
       <c r="F11" t="str">
-        <v>Collectible desk dragon for fantasy fans. Inspired by iconic TV series dragons.</v>
+        <v>Collectible desk guardian for those who understand that dragons were never just stories.</v>
       </c>
       <c r="G11" t="str">
         <v>Collectibles</v>
       </c>
       <c r="H11" t="str">
-        <v>https://placeholder-image-url.com/dragon.jpg</v>
+        <v>https://placeholder-image-url.com/mythic-serpent.jpg</v>
       </c>
       <c r="I11" t="str">
         <v>18cm x 8cm x 6cm</v>
@@ -756,10 +756,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>Batman Logo Desk Organizer</v>
+        <v>Night Guardian Desk Organizer</v>
       </c>
       <c r="C12" t="str">
-        <v>Laser-cut black acrylic desk organizer shaped like the Batman symbol. Multiple compartments for pens and cards.</v>
+        <v>Laser-cut black acrylic desk organizer shaped like a winged emblem. Multiple compartments for pens and cards. Darkness as design. Justice as aesthetic.</v>
       </c>
       <c r="D12">
         <v>799</v>
@@ -768,13 +768,13 @@
         <v>Black Acrylic</v>
       </c>
       <c r="F12" t="str">
-        <v>Bring Gotham to your desk. Perfect for DC Comics fans who want subtle, stylish merchandise.</v>
+        <v>Bring Gotham-level organization to your workspace. For vigilantes of productivity.</v>
       </c>
       <c r="G12" t="str">
         <v>Desk Accessories</v>
       </c>
       <c r="H12" t="str">
-        <v>https://placeholder-image-url.com/batman.jpg</v>
+        <v>https://placeholder-image-url.com/night-guardian.jpg</v>
       </c>
       <c r="I12" t="str">
         <v>20cm x 10cm x 8cm</v>
@@ -788,10 +788,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>Anime Character Keychain Set</v>
+        <v>Character Totem Keychain Set</v>
       </c>
       <c r="C13" t="str">
-        <v>Set of 3 custom 3D-printed keychains. Popular anime character silhouettes with vibrant colors.</v>
+        <v>Set of 3 custom 3D-printed keychains. Eastern animation character silhouettes with vibrant colors. Carry your universe wherever you go.</v>
       </c>
       <c r="D13">
         <v>399</v>
@@ -800,13 +800,13 @@
         <v>PETG Plastic</v>
       </c>
       <c r="F13" t="str">
-        <v>Show your anime love on your keys or bag. Makes a great gift for anime fans.</v>
+        <v>Identity on your keys. For those whose worlds are not limited by geography or medium.</v>
       </c>
       <c r="G13" t="str">
         <v>Gifts</v>
       </c>
       <c r="H13" t="str">
-        <v>https://placeholder-image-url.com/anime-keychain.jpg</v>
+        <v>https://placeholder-image-url.com/character-totem.jpg</v>
       </c>
       <c r="I13" t="str">
         <v>5cm x 3cm x 0.5cm (each)</v>
@@ -820,10 +820,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>Mjolnir (Thor's Hammer) Paperweight</v>
+        <v>Thunder Relic Paperweight</v>
       </c>
       <c r="C14" t="str">
-        <v>3D-printed replica of Thor's hammer. Heavy enough to serve as a functional paperweight.</v>
+        <v>3D-printed replica of a legendary hammer. Heavy enough to hold down your papers, symbolic enough to declare worthiness. Are you worthy? Your desk will answer.</v>
       </c>
       <c r="D14">
         <v>699</v>
@@ -832,13 +832,13 @@
         <v>PLA Plastic with Metal Fill</v>
       </c>
       <c r="F14" t="str">
-        <v>Are you worthy? This Mjolnir paperweight keeps your papers in place, Marvel style.</v>
+        <v>Papers stay down. Thunder stays up. For those who wield responsibility with power.</v>
       </c>
       <c r="G14" t="str">
         <v>Desk Accessories</v>
       </c>
       <c r="H14" t="str">
-        <v>https://placeholder-image-url.com/mjolnir.jpg</v>
+        <v>https://placeholder-image-url.com/thunder-relic.jpg</v>
       </c>
       <c r="I14" t="str">
         <v>12cm x 8cm x 6cm</v>
@@ -852,10 +852,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>Golden Snitch Desk Sculpture</v>
+        <v>Winged Quest Desk Sculpture</v>
       </c>
       <c r="C15" t="str">
-        <v>3D-printed Golden Snitch with delicate wings. Can be placed on your desk or hung as decoration.</v>
+        <v>3D-printed golden sphere with delicate wings. Can be placed or hung. The hardest to catch, the most precious to hold. Seeker pride in tangible form.</v>
       </c>
       <c r="D15">
         <v>599</v>
@@ -864,13 +864,13 @@
         <v>Gold PLA Plastic</v>
       </c>
       <c r="F15" t="str">
-        <v>Catch this Snitch for your desk. Perfect for Quidditch fans and Potterheads.</v>
+        <v>For those who chase impossible things until they become real. Crafted in Jaipur.</v>
       </c>
       <c r="G15" t="str">
         <v>Collectibles</v>
       </c>
       <c r="H15" t="str">
-        <v>https://placeholder-image-url.com/snitch.jpg</v>
+        <v>https://placeholder-image-url.com/winged-quest.jpg</v>
       </c>
       <c r="I15" t="str">
         <v>8cm wingspan x 4cm</v>
@@ -884,10 +884,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>Customized Fandom Quote Plaque</v>
+        <v>Universe Echo Quote Plaque</v>
       </c>
       <c r="C16" t="str">
-        <v>Laser-cut wooden plaque with your favorite fandom quote. Choose from HP, Marvel, Star Wars, or custom text.</v>
+        <v>Laser-cut wooden plaque with your chosen quote from any universe. Wizarding world, superhero sagas, galactic epics, or your own words. Your philosophy, made permanent.</v>
       </c>
       <c r="D16">
         <v>749</v>
@@ -896,13 +896,13 @@
         <v>Oak Wood</v>
       </c>
       <c r="F16" t="str">
-        <v>Display your favorite quote from any fandom. Perfect personalized gift for fans.</v>
+        <v>Words that define you, carved in wood. Personalized identity artifact. Crafted in Jaipur.</v>
       </c>
       <c r="G16" t="str">
         <v>Gifts</v>
       </c>
       <c r="H16" t="str">
-        <v>https://placeholder-image-url.com/quote-plaque.jpg</v>
+        <v>https://placeholder-image-url.com/universe-echo.jpg</v>
       </c>
       <c r="I16" t="str">
         <v>25cm x 15cm x 1cm</v>

</xml_diff>

<commit_message>
Removed categories from frontend. Made grid
</commit_message>
<xml_diff>
--- a/server/data/products.xlsx
+++ b/server/data/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -815,105 +815,9 @@
         <v>15g (each)</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Thunder Relic Paperweight</v>
-      </c>
-      <c r="C14" t="str">
-        <v>3D-printed replica of a legendary hammer. Heavy enough to hold down your papers, symbolic enough to declare worthiness. Are you worthy? Your desk will answer.</v>
-      </c>
-      <c r="D14">
-        <v>699</v>
-      </c>
-      <c r="E14" t="str">
-        <v>PLA Plastic with Metal Fill</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Papers stay down. Thunder stays up. For those who wield responsibility with power.</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Desk Accessories</v>
-      </c>
-      <c r="H14" t="str">
-        <v>https://placeholder-image-url.com/thunder-relic.jpg</v>
-      </c>
-      <c r="I14" t="str">
-        <v>12cm x 8cm x 6cm</v>
-      </c>
-      <c r="J14" t="str">
-        <v>200g</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Winged Quest Desk Sculpture</v>
-      </c>
-      <c r="C15" t="str">
-        <v>3D-printed golden sphere with delicate wings. Can be placed or hung. The hardest to catch, the most precious to hold. Seeker pride in tangible form.</v>
-      </c>
-      <c r="D15">
-        <v>599</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Gold PLA Plastic</v>
-      </c>
-      <c r="F15" t="str">
-        <v>For those who chase impossible things until they become real. Crafted in Jaipur.</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Collectibles</v>
-      </c>
-      <c r="H15" t="str">
-        <v>https://placeholder-image-url.com/winged-quest.jpg</v>
-      </c>
-      <c r="I15" t="str">
-        <v>8cm wingspan x 4cm</v>
-      </c>
-      <c r="J15" t="str">
-        <v>25g</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Universe Echo Quote Plaque</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Laser-cut wooden plaque with your chosen quote from any universe. Wizarding world, superhero sagas, galactic epics, or your own words. Your philosophy, made permanent.</v>
-      </c>
-      <c r="D16">
-        <v>749</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Oak Wood</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Words that define you, carved in wood. Personalized identity artifact. Crafted in Jaipur.</v>
-      </c>
-      <c r="G16" t="str">
-        <v>Gifts</v>
-      </c>
-      <c r="H16" t="str">
-        <v>https://placeholder-image-url.com/universe-echo.jpg</v>
-      </c>
-      <c r="I16" t="str">
-        <v>25cm x 15cm x 1cm</v>
-      </c>
-      <c r="J16" t="str">
-        <v>180g</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added product images, updated generateExcel.js Fixed footer Fixed contact section Commented dimentions and weight in product details
</commit_message>
<xml_diff>
--- a/server/data/products.xlsx
+++ b/server/data/products.xlsx
@@ -436,31 +436,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>House Sigil Desk Monument</v>
+        <v>Thing Hand</v>
       </c>
       <c r="C2" t="str">
-        <v>Four ancient houses. One choice that defines you. Laser-cut wooden monument featuring your chosen sigil. For those who know that where you belong matters more than where you started. Precision-crafted in Jaipur.</v>
+        <v>3D-printed replica of Thing from Wednesday, designed as a collectible desk artifact for fans of the series.</v>
       </c>
       <c r="D2">
-        <v>899</v>
+        <v>600</v>
       </c>
       <c r="E2" t="str">
-        <v>Birch Wood</v>
+        <v>PLA</v>
       </c>
       <c r="F2" t="str">
-        <v>Declare your allegiance. Symbol of wisdom, courage, ambition, or loyalty - your desk, your manifesto.</v>
+        <v>Display on a desk, shelf, or fandom corner as a collectible prop.</v>
       </c>
       <c r="G2" t="str">
         <v>Collectibles</v>
       </c>
       <c r="H2" t="str">
-        <v>https://placeholder-image-url.com/house-sigil.jpg</v>
+        <v>/products/thing/thing.JPG</v>
       </c>
       <c r="I2" t="str">
-        <v>15cm x 12cm x 3cm</v>
+        <v>10cm x 8cm x 6cm</v>
       </c>
       <c r="J2" t="str">
-        <v>120g</v>
+        <v>90g</v>
       </c>
     </row>
     <row r="3">
@@ -468,31 +468,31 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Arc Emblem Phone Stand</v>
+        <v>Max Bookmark</v>
       </c>
       <c r="C3" t="str">
-        <v>3D-printed phone stand inspired by genius engineering. Power symbol in circular precision. Holds your device at the perfect angle. For those who know innovation is identity.</v>
+        <v>Stranger Things inspired bookmark themed around Max, made for readers who love the series.</v>
       </c>
       <c r="D3">
-        <v>749</v>
+        <v>180</v>
       </c>
       <c r="E3" t="str">
-        <v>PLA Plastic</v>
+        <v>PLA</v>
       </c>
       <c r="F3" t="str">
-        <v>Your workspace, powered by the same energy that drives visionaries. Precision-cut in Jaipur.</v>
+        <v>Bookmark for novels, journals, and fandom collections.</v>
       </c>
       <c r="G3" t="str">
-        <v>Desk Accessories</v>
+        <v>Bookmarks</v>
       </c>
       <c r="H3" t="str">
-        <v>https://placeholder-image-url.com/arc-emblem.jpg</v>
+        <v>/products/st-bm/st-bm.JPG</v>
       </c>
       <c r="I3" t="str">
-        <v>12cm x 10cm x 8cm</v>
+        <v>15cm x 4cm x 0.3cm</v>
       </c>
       <c r="J3" t="str">
-        <v>95g</v>
+        <v>12g</v>
       </c>
     </row>
     <row r="4">
@@ -500,31 +500,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Dueling Relic Pen Holder</v>
+        <v>Harry Potter Bookmark 1</v>
       </c>
       <c r="C4" t="str">
-        <v>Laser-cut acrylic pen holder shaped like an elegant weapon hilt. Choose your allegiance: guardian blue or defiant red. Ancient conflicts, modern desk. The Force is not fiction - it is philosophy.</v>
+        <v>Harry Potter inspired bookmark designed for fans who want a magical touch while reading.</v>
       </c>
       <c r="D4">
-        <v>649</v>
+        <v>100</v>
       </c>
       <c r="E4" t="str">
-        <v>Colored Acrylic</v>
+        <v>PLA</v>
       </c>
       <c r="F4" t="str">
-        <v>Store your tools in a symbol of cosmic balance. Light or dark - your choice, your identity.</v>
+        <v>Use while reading books or keep as a collectible fandom accessory.</v>
       </c>
       <c r="G4" t="str">
-        <v>Desk Accessories</v>
+        <v>Bookmarks</v>
       </c>
       <c r="H4" t="str">
-        <v>https://placeholder-image-url.com/dueling-relic.jpg</v>
+        <v>/products/hp-bm1/hp-bm1.JPG</v>
       </c>
       <c r="I4" t="str">
-        <v>20cm x 5cm x 5cm</v>
+        <v>15cm x 4cm x 0.3cm</v>
       </c>
       <c r="J4" t="str">
-        <v>80g</v>
+        <v>12g</v>
       </c>
     </row>
     <row r="5">
@@ -532,31 +532,31 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Cosmic Script Name Plate</v>
+        <v>Harry Potter Bookmark 2</v>
       </c>
       <c r="C5" t="str">
-        <v>Laser-cut wooden name plate with your name in an otherworldly font, complete with star accents. Custom engraving. Professional, yet subtly extraordinary. Crafted in Jaipur.</v>
+        <v>Second Harry Potter inspired bookmark with a magical fandom theme, suitable for readers and collectors.</v>
       </c>
       <c r="D5">
-        <v>599</v>
+        <v>125</v>
       </c>
       <c r="E5" t="str">
-        <v>Walnut Wood</v>
+        <v>PLA</v>
       </c>
       <c r="F5" t="str">
-        <v>Your name, your desk, your universe. For those who bring magic to the mundane without explanation.</v>
+        <v>Bookmark for books and a collectible add-on for Harry Potter fans.</v>
       </c>
       <c r="G5" t="str">
-        <v>Gifts</v>
+        <v>Bookmarks</v>
       </c>
       <c r="H5" t="str">
-        <v>https://placeholder-image-url.com/cosmic-nameplate.jpg</v>
+        <v>/products/hp-bm2/hp-bm2.JPG</v>
       </c>
       <c r="I5" t="str">
-        <v>22cm x 6cm x 1.5cm</v>
+        <v>15cm x 4cm x 0.3cm</v>
       </c>
       <c r="J5" t="str">
-        <v>90g</v>
+        <v>12g</v>
       </c>
     </row>
     <row r="6">
@@ -564,31 +564,31 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>Hero Emblems Coaster Set</v>
+        <v>Golden Snitch</v>
       </c>
       <c r="C6" t="str">
-        <v>Set of 4 laser-cut wooden coasters featuring iconic superhero symbols. Shield, arc, lightning, strength. Protect your desk surface while quietly declaring allegiance to extraordinary ideals.</v>
+        <v>3D-printed Golden Snitch inspired by Harry Potter, made as a collectible decorative artifact.</v>
       </c>
       <c r="D6">
-        <v>499</v>
+        <v>350</v>
       </c>
       <c r="E6" t="str">
-        <v>Bamboo Wood</v>
+        <v>PLA</v>
       </c>
       <c r="F6" t="str">
-        <v>Not all heroes wear capes. Some just have impeccable desk aesthetics. Indian-crafted precision.</v>
+        <v>Display piece for shelves, desks, and fandom setups.</v>
       </c>
       <c r="G6" t="str">
-        <v>Desk Accessories</v>
+        <v>Collectibles</v>
       </c>
       <c r="H6" t="str">
-        <v>https://placeholder-image-url.com/hero-emblems.jpg</v>
+        <v>/products/snitch-ball/snitch-ball.JPG</v>
       </c>
       <c r="I6" t="str">
-        <v>10cm diameter x 0.8cm (each)</v>
+        <v>8cm x 12cm x 8cm</v>
       </c>
       <c r="J6" t="str">
-        <v>40g (each)</v>
+        <v>35g</v>
       </c>
     </row>
     <row r="7">
@@ -596,31 +596,31 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>Small Guardian Desk Companion</v>
+        <v>Sorting Hat</v>
       </c>
       <c r="C7" t="str">
-        <v>3D-printed desk companion with large, knowing eyes. Adorable design with precise detailing. Watches over your workspace with ancient wisdom in tiny form. This is the way.</v>
+        <v>Harry Potter inspired Sorting Hat model, recreated as a detailed collectible for fans.</v>
       </c>
       <c r="D7">
-        <v>999</v>
+        <v>250</v>
       </c>
       <c r="E7" t="str">
-        <v>PLA Plastic</v>
+        <v>PLA</v>
       </c>
       <c r="F7" t="str">
-        <v>Desk guardian for those who understand that the most powerful often come in unexpected packages.</v>
+        <v>Decor item for desks, bookshelves, and fandom collections.</v>
       </c>
       <c r="G7" t="str">
         <v>Collectibles</v>
       </c>
       <c r="H7" t="str">
-        <v>https://placeholder-image-url.com/guardian.jpg</v>
+        <v>/products/sorting-hat/sorting-hat.JPG</v>
       </c>
       <c r="I7" t="str">
-        <v>10cm x 6cm x 6cm</v>
+        <v>11cm x 11cm x 9cm</v>
       </c>
       <c r="J7" t="str">
-        <v>75g</v>
+        <v>85g</v>
       </c>
     </row>
     <row r="8">
@@ -628,31 +628,31 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>Wisdom Keeper Pen Stand</v>
+        <v>Nimbus 2000</v>
       </c>
       <c r="C8" t="str">
-        <v>3D-printed replica of an ancient sorting artifact that holds your pens. Detailed texture and weathered finish. Let destiny decide where your tools belong.</v>
+        <v>Harry Potter inspired Nimbus 2000 miniature, created as a decorative collectible prop.</v>
       </c>
       <c r="D8">
-        <v>849</v>
+        <v>900</v>
       </c>
       <c r="E8" t="str">
-        <v>PLA Plastic</v>
+        <v>PLA</v>
       </c>
       <c r="F8" t="str">
-        <v>Organize your stationery with the same wisdom that sorts souls. Crafted in Jaipur workshops.</v>
+        <v>Display as a miniature prop on desks, stands, or themed setups.</v>
       </c>
       <c r="G8" t="str">
-        <v>Desk Accessories</v>
+        <v>Collectibles</v>
       </c>
       <c r="H8" t="str">
-        <v>https://placeholder-image-url.com/wisdom-keeper.jpg</v>
+        <v>/products/nimbus/nimbus.JPG</v>
       </c>
       <c r="I8" t="str">
-        <v>12cm x 12cm x 10cm</v>
+        <v>20cm x 3cm x 4cm</v>
       </c>
       <c r="J8" t="str">
-        <v>110g</v>
+        <v>40g</v>
       </c>
     </row>
     <row r="9">
@@ -660,31 +660,31 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Arachnid Web Cable Organizer</v>
+        <v>Demadog</v>
       </c>
       <c r="C9" t="str">
-        <v>3D-printed cable holder inspired by bio-mechanical precision. Keeps your desk cables tangle-free with spider-like efficiency. With great organization comes great productivity.</v>
+        <v>Stranger Things inspired Demadog figure, made as a detailed collectible for fans of the Upside Down.</v>
       </c>
       <c r="D9">
-        <v>449</v>
+        <v>300</v>
       </c>
       <c r="E9" t="str">
-        <v>PLA Plastic</v>
+        <v>PLA</v>
       </c>
       <c r="F9" t="str">
-        <v>Web-slinging cable management for those who swing between chaos and control. Set of 2.</v>
+        <v>Collectible display model for desks, shelves, and themed rooms.</v>
       </c>
       <c r="G9" t="str">
-        <v>Desk Accessories</v>
+        <v>Collectibles</v>
       </c>
       <c r="H9" t="str">
-        <v>https://placeholder-image-url.com/web-organizer.jpg</v>
+        <v>/products/demadog/demadog.JPG</v>
       </c>
       <c r="I9" t="str">
-        <v>6cm x 4cm x 3cm (each)</v>
+        <v>14cm x 8cm x 7cm</v>
       </c>
       <c r="J9" t="str">
-        <v>30g (each)</v>
+        <v>95g</v>
       </c>
     </row>
     <row r="10">
@@ -692,31 +692,31 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Hallowed Symbols Bookmark</v>
+        <v>Deathly Hallows Frame</v>
       </c>
       <c r="C10" t="str">
-        <v>Laser-cut wooden bookmark featuring the trinity of ancient relics. Elegant and meaningful. Three objects, one master of death. Mark your place in stories that matter.</v>
+        <v>Harry Potter inspired decorative frame featuring the Deathly Hallows symbol.</v>
       </c>
       <c r="D10">
-        <v>249</v>
+        <v>300</v>
       </c>
       <c r="E10" t="str">
-        <v>Walnut Wood</v>
+        <v>PLA</v>
       </c>
       <c r="F10" t="str">
-        <v>For readers who know that some symbols hold more power than words. Indian-crafted precision.</v>
+        <v>Wall or shelf decor piece for fandom spaces and personal collections.</v>
       </c>
       <c r="G10" t="str">
-        <v>Gifts</v>
+        <v>Decor</v>
       </c>
       <c r="H10" t="str">
-        <v>https://placeholder-image-url.com/hallowed-symbols.jpg</v>
+        <v>/products/wall-hanging/wall-hanging.JPG</v>
       </c>
       <c r="I10" t="str">
-        <v>15cm x 4cm x 0.3cm</v>
+        <v>18cm x 18cm x 1.5cm</v>
       </c>
       <c r="J10" t="str">
-        <v>10g</v>
+        <v>120g</v>
       </c>
     </row>
     <row r="11">
@@ -724,31 +724,31 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Articulated Mythic Serpent</v>
+        <v>Iron Throne</v>
       </c>
       <c r="C11" t="str">
-        <v>3D-printed articulated creature with movable wings and body. Fully poseable with smooth joints. Fantasy made tangible. Fire and flight in flexible form.</v>
+        <v>Game of Thrones inspired Iron Throne model, recreated as a collectible display artifact.</v>
       </c>
       <c r="D11">
-        <v>999</v>
+        <v>800</v>
       </c>
       <c r="E11" t="str">
-        <v>TPU Flexible Plastic</v>
+        <v>PLA</v>
       </c>
       <c r="F11" t="str">
-        <v>Collectible desk guardian for those who understand that dragons were never just stories.</v>
+        <v>Premium collectible for desk display, shelf decor, or themed setups.</v>
       </c>
       <c r="G11" t="str">
         <v>Collectibles</v>
       </c>
       <c r="H11" t="str">
-        <v>https://placeholder-image-url.com/mythic-serpent.jpg</v>
+        <v>/products/throne/throne.JPG</v>
       </c>
       <c r="I11" t="str">
-        <v>18cm x 8cm x 6cm</v>
+        <v>16cm x 10cm x 8cm</v>
       </c>
       <c r="J11" t="str">
-        <v>110g</v>
+        <v>150g</v>
       </c>
     </row>
     <row r="12">
@@ -756,31 +756,31 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>Night Guardian Desk Organizer</v>
+        <v>Golden Snitch Book Page Holder</v>
       </c>
       <c r="C12" t="str">
-        <v>Laser-cut black acrylic desk organizer shaped like a winged emblem. Multiple compartments for pens and cards. Darkness as design. Justice as aesthetic.</v>
+        <v>Harry Potter inspired book page holder with Golden Snitch theme, designed for readers and collectors.</v>
       </c>
       <c r="D12">
-        <v>799</v>
+        <v>150</v>
       </c>
       <c r="E12" t="str">
-        <v>Black Acrylic</v>
+        <v>PLA</v>
       </c>
       <c r="F12" t="str">
-        <v>Bring Gotham-level organization to your workspace. For vigilantes of productivity.</v>
+        <v>Hold book pages open while reading and serve as a fandom accessory.</v>
       </c>
       <c r="G12" t="str">
-        <v>Desk Accessories</v>
+        <v>Book Accessories</v>
       </c>
       <c r="H12" t="str">
-        <v>https://placeholder-image-url.com/night-guardian.jpg</v>
+        <v>/products/snitch-bh/snitch-bh.JPG</v>
       </c>
       <c r="I12" t="str">
-        <v>20cm x 10cm x 8cm</v>
+        <v>7cm x 7cm x 2cm</v>
       </c>
       <c r="J12" t="str">
-        <v>150g</v>
+        <v>25g</v>
       </c>
     </row>
     <row r="13">
@@ -788,31 +788,31 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>Character Totem Keychain Set</v>
+        <v>Groot</v>
       </c>
       <c r="C13" t="str">
-        <v>Set of 3 custom 3D-printed keychains. Eastern animation character silhouettes with vibrant colors. Carry your universe wherever you go.</v>
+        <v>Marvel inspired Groot figure, made as a decorative collectible for superhero fans.</v>
       </c>
       <c r="D13">
-        <v>399</v>
+        <v>450</v>
       </c>
       <c r="E13" t="str">
-        <v>PETG Plastic</v>
+        <v>PLA</v>
       </c>
       <c r="F13" t="str">
-        <v>Identity on your keys. For those whose worlds are not limited by geography or medium.</v>
+        <v>Display on desks, shelves, or gift to Marvel fans.</v>
       </c>
       <c r="G13" t="str">
-        <v>Gifts</v>
+        <v>Collectibles</v>
       </c>
       <c r="H13" t="str">
-        <v>https://placeholder-image-url.com/character-totem.jpg</v>
+        <v>/products/groot/groot.JPG</v>
       </c>
       <c r="I13" t="str">
-        <v>5cm x 3cm x 0.5cm (each)</v>
+        <v>12cm x 7cm x 7cm</v>
       </c>
       <c r="J13" t="str">
-        <v>15g (each)</v>
+        <v>80g</v>
       </c>
     </row>
   </sheetData>

</xml_diff>